<commit_message>
feat: single-page PDF, bulk download (all/range/custom), mode tabs UI
</commit_message>
<xml_diff>
--- a/uploads/applicants.xlsx
+++ b/uploads/applicants.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6493" uniqueCount="2575">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6513" uniqueCount="2586">
   <si>
     <t>Timestamp</t>
   </si>
@@ -7743,6 +7743,39 @@
   </si>
   <si>
     <t xml:space="preserve">ANAS PLASTIC </t>
+  </si>
+  <si>
+    <t>42301-6356178-3</t>
+  </si>
+  <si>
+    <t>Ussama</t>
+  </si>
+  <si>
+    <t>AYUB</t>
+  </si>
+  <si>
+    <t>Muhammad Ayub</t>
+  </si>
+  <si>
+    <t>AT1131782</t>
+  </si>
+  <si>
+    <t>Flat No5 3rd floor Al-Qamar Mansion burns road south karachi</t>
+  </si>
+  <si>
+    <t>03212700164</t>
+  </si>
+  <si>
+    <t>42301-3447241-5</t>
+  </si>
+  <si>
+    <t>03222505075</t>
+  </si>
+  <si>
+    <t>PK04MEZN0001640103475205</t>
+  </si>
+  <si>
+    <t>USSAMA</t>
   </si>
 </sst>
 </file>
@@ -7904,7 +7937,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:AB354" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:AB355" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="28">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Family Size  " id="2"/>
@@ -8259,26 +8292,26 @@
       </c>
       <c r="C2" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("ARRAYFORMULA(
-IF(D2:D453="""","""",
-IF(UPPER(TRIM(F2:F453))=""SHORT"",""S"",""L"")&amp;
+IF(D2:D454="""","""",
+IF(UPPER(TRIM(F2:F454))=""SHORT"",""S"",""L"")&amp;
 IF(
-UPPER(TRIM(F2:F453))=""SHORT"",
+UPPER(TRIM(F2:F454))=""SHORT"",
 MATCH(
-REGEXREPLACE(TO_TEXT(D2:D453),""[^0-9]"",""""),
+REGEXREPLACE(TO_TEXT(D2:D454),""[^0-9]"",""""),
 UNIQUE(
 FILTER(
-REGEXREPLACE(TO_TEXT(D2:D453),""[^0-9]"",""""),
-(D2:D453&lt;&gt;"""")*"&amp;"(UPPER(TRIM(F2:F453))=""SHORT"")
+REGEXREPLACE(TO_TEXT(D2:D454),""[^0-9]"",""""),
+(D2:D454&lt;&gt;"""")*"&amp;"(UPPER(TRIM(F2:F454))=""SHORT"")
 )
 ),
 0
 ),
 MATCH(
-REGEXREPLACE(TO_TEXT(D2:D453),""[^0-9]"",""""),
+REGEXREPLACE(TO_TEXT(D2:D454),""[^0-9]"",""""),
 UNIQUE(
 FILTER(
-REGEXREPLACE(TO_TEXT(D2:D453),""[^0-9]"",""""),
-(D2:D453&lt;&gt;"""")*(UPPER(TRIM(F2:F453))=""LONG"")
+REGEXREPLACE(TO_TEXT(D2:D454),""[^0-9]"",""""),
+(D2:D454&lt;&gt;"""")*(UPPER(TRIM(F2:F454))=""LONG"")
 )
 ),
 0
@@ -36079,43 +36112,115 @@
       </c>
     </row>
     <row r="354" ht="22.5" customHeight="1">
-      <c r="A354" s="10"/>
-      <c r="B354" s="10"/>
-      <c r="C354" s="10" t="str">
+      <c r="A354" s="3">
+        <v>46210.40233092592</v>
+      </c>
+      <c r="B354" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="C354" s="5" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"L88")</f>
+        <v>L88</v>
+      </c>
+      <c r="D354" s="4" t="s">
+        <v>2575</v>
+      </c>
+      <c r="E354" s="4" t="s">
+        <v>2576</v>
+      </c>
+      <c r="F354" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G354" s="4" t="s">
+        <v>2577</v>
+      </c>
+      <c r="H354" s="4" t="s">
+        <v>2576</v>
+      </c>
+      <c r="I354" s="4" t="s">
+        <v>2578</v>
+      </c>
+      <c r="J354" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="K354" s="4" t="s">
+        <v>2579</v>
+      </c>
+      <c r="L354" s="6">
+        <v>49840.0</v>
+      </c>
+      <c r="M354" s="4" t="s">
+        <v>2575</v>
+      </c>
+      <c r="N354" s="6">
+        <v>34429.0</v>
+      </c>
+      <c r="O354" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="P354" s="4" t="s">
+        <v>2580</v>
+      </c>
+      <c r="Q354" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="R354" s="7" t="s">
+        <v>2581</v>
+      </c>
+      <c r="S354" s="7" t="s">
+        <v>2581</v>
+      </c>
+      <c r="V354" s="4" t="s">
+        <v>2578</v>
+      </c>
+      <c r="W354" s="4" t="s">
+        <v>2582</v>
+      </c>
+      <c r="X354" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y354" s="7" t="s">
+        <v>2583</v>
+      </c>
+      <c r="Z354" s="4" t="s">
+        <v>2584</v>
+      </c>
+      <c r="AA354" s="4" t="s">
+        <v>2585</v>
+      </c>
+    </row>
+    <row r="355" ht="22.5" customHeight="1">
+      <c r="A355" s="10"/>
+      <c r="B355" s="10"/>
+      <c r="C355" s="10" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
         <v/>
       </c>
-      <c r="D354" s="10"/>
-      <c r="E354" s="10"/>
-      <c r="F354" s="10"/>
-      <c r="G354" s="10"/>
-      <c r="H354" s="10"/>
-      <c r="I354" s="10"/>
-      <c r="J354" s="10"/>
-      <c r="K354" s="10"/>
-      <c r="L354" s="10"/>
-      <c r="M354" s="10"/>
-      <c r="N354" s="10"/>
-      <c r="O354" s="10"/>
-      <c r="P354" s="10"/>
-      <c r="Q354" s="10"/>
-      <c r="R354" s="10"/>
-      <c r="S354" s="10"/>
-      <c r="T354" s="10"/>
-      <c r="U354" s="10"/>
-      <c r="V354" s="10"/>
-      <c r="W354" s="10"/>
-      <c r="X354" s="10"/>
-      <c r="Y354" s="10"/>
-      <c r="Z354" s="10"/>
-      <c r="AA354" s="10"/>
-      <c r="AB354" s="10"/>
-    </row>
-    <row r="355">
-      <c r="C355" s="11" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
-        <v/>
-      </c>
+      <c r="D355" s="10"/>
+      <c r="E355" s="10"/>
+      <c r="F355" s="10"/>
+      <c r="G355" s="10"/>
+      <c r="H355" s="10"/>
+      <c r="I355" s="10"/>
+      <c r="J355" s="10"/>
+      <c r="K355" s="10"/>
+      <c r="L355" s="10"/>
+      <c r="M355" s="10"/>
+      <c r="N355" s="10"/>
+      <c r="O355" s="10"/>
+      <c r="P355" s="10"/>
+      <c r="Q355" s="10"/>
+      <c r="R355" s="10"/>
+      <c r="S355" s="10"/>
+      <c r="T355" s="10"/>
+      <c r="U355" s="10"/>
+      <c r="V355" s="10"/>
+      <c r="W355" s="10"/>
+      <c r="X355" s="10"/>
+      <c r="Y355" s="10"/>
+      <c r="Z355" s="10"/>
+      <c r="AA355" s="10"/>
+      <c r="AB355" s="10"/>
     </row>
     <row r="356">
       <c r="C356" s="11" t="str">
@@ -36701,6 +36806,12 @@
     </row>
     <row r="453">
       <c r="C453" s="11" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="454">
+      <c r="C454" s="11" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
fix: wrap thread pool workers with app.app_context() to allow render_template
</commit_message>
<xml_diff>
--- a/uploads/applicants.xlsx
+++ b/uploads/applicants.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6513" uniqueCount="2586">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6572" uniqueCount="2613">
   <si>
     <t>Timestamp</t>
   </si>
@@ -7776,6 +7776,87 @@
   </si>
   <si>
     <t>USSAMA</t>
+  </si>
+  <si>
+    <t>42201-1642171-5</t>
+  </si>
+  <si>
+    <t>Muhammad Rasim Qureshi</t>
+  </si>
+  <si>
+    <t>Aleem</t>
+  </si>
+  <si>
+    <t>Khudaija Aleem</t>
+  </si>
+  <si>
+    <t>Muhammad Aleem Qureshi</t>
+  </si>
+  <si>
+    <t>42201-0643261-4</t>
+  </si>
+  <si>
+    <t>L-649 Sector 2 North Karachi.</t>
+  </si>
+  <si>
+    <t>92332- 8278682</t>
+  </si>
+  <si>
+    <t>0332- 8278682</t>
+  </si>
+  <si>
+    <t>Muhammad Zunair Qureshi</t>
+  </si>
+  <si>
+    <t>42201-2545997-3</t>
+  </si>
+  <si>
+    <t>0335-7596636</t>
+  </si>
+  <si>
+    <t>01080107517815</t>
+  </si>
+  <si>
+    <t>42401-8841192-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abdul Munaf </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mohammed </t>
+  </si>
+  <si>
+    <t>AE0781922</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khawja gareeb Nawaz heights 2nd floor front portion plot no 4/23 nazmabad no 3b </t>
+  </si>
+  <si>
+    <t>03218793525</t>
+  </si>
+  <si>
+    <t>42301-9698364-6</t>
+  </si>
+  <si>
+    <t>03222508056</t>
+  </si>
+  <si>
+    <t>Pk35BAHL1182182500860601</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sadia </t>
+  </si>
+  <si>
+    <t>Qureshi</t>
+  </si>
+  <si>
+    <t>L-649 SECTOR 2 North Karachi.</t>
+  </si>
+  <si>
+    <t>0327-2510491</t>
+  </si>
+  <si>
+    <t>MUHAMMAD RASIM QURESHI</t>
   </si>
 </sst>
 </file>
@@ -7937,7 +8018,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:AB355" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:AB358" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="28">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Family Size  " id="2"/>
@@ -8292,26 +8373,26 @@
       </c>
       <c r="C2" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("ARRAYFORMULA(
-IF(D2:D454="""","""",
-IF(UPPER(TRIM(F2:F454))=""SHORT"",""S"",""L"")&amp;
+IF(D2:D457="""","""",
+IF(UPPER(TRIM(F2:F457))=""SHORT"",""S"",""L"")&amp;
 IF(
-UPPER(TRIM(F2:F454))=""SHORT"",
+UPPER(TRIM(F2:F457))=""SHORT"",
 MATCH(
-REGEXREPLACE(TO_TEXT(D2:D454),""[^0-9]"",""""),
+REGEXREPLACE(TO_TEXT(D2:D457),""[^0-9]"",""""),
 UNIQUE(
 FILTER(
-REGEXREPLACE(TO_TEXT(D2:D454),""[^0-9]"",""""),
-(D2:D454&lt;&gt;"""")*"&amp;"(UPPER(TRIM(F2:F454))=""SHORT"")
+REGEXREPLACE(TO_TEXT(D2:D457),""[^0-9]"",""""),
+(D2:D457&lt;&gt;"""")*"&amp;"(UPPER(TRIM(F2:F457))=""SHORT"")
 )
 ),
 0
 ),
 MATCH(
-REGEXREPLACE(TO_TEXT(D2:D454),""[^0-9]"",""""),
+REGEXREPLACE(TO_TEXT(D2:D457),""[^0-9]"",""""),
 UNIQUE(
 FILTER(
-REGEXREPLACE(TO_TEXT(D2:D454),""[^0-9]"",""""),
-(D2:D454&lt;&gt;"""")*(UPPER(TRIM(F2:F454))=""LONG"")
+REGEXREPLACE(TO_TEXT(D2:D457),""[^0-9]"",""""),
+(D2:D457&lt;&gt;"""")*(UPPER(TRIM(F2:F457))=""LONG"")
 )
 ),
 0
@@ -36190,55 +36271,265 @@
       </c>
     </row>
     <row r="355" ht="22.5" customHeight="1">
-      <c r="A355" s="10"/>
-      <c r="B355" s="10"/>
-      <c r="C355" s="10" t="str">
+      <c r="A355" s="3">
+        <v>46210.54221767361</v>
+      </c>
+      <c r="B355" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="C355" s="5" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"L89")</f>
+        <v>L89</v>
+      </c>
+      <c r="D355" s="4" t="s">
+        <v>2586</v>
+      </c>
+      <c r="E355" s="4" t="s">
+        <v>2587</v>
+      </c>
+      <c r="F355" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G355" s="4" t="s">
+        <v>2588</v>
+      </c>
+      <c r="H355" s="4" t="s">
+        <v>2589</v>
+      </c>
+      <c r="I355" s="4" t="s">
+        <v>2590</v>
+      </c>
+      <c r="J355" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="M355" s="4" t="s">
+        <v>2591</v>
+      </c>
+      <c r="N355" s="6">
+        <v>29106.0</v>
+      </c>
+      <c r="O355" s="4" t="s">
+        <v>1597</v>
+      </c>
+      <c r="P355" s="4" t="s">
+        <v>2592</v>
+      </c>
+      <c r="Q355" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="R355" s="4" t="s">
+        <v>2593</v>
+      </c>
+      <c r="S355" s="4" t="s">
+        <v>2594</v>
+      </c>
+      <c r="T355" s="4" t="s">
+        <v>2587</v>
+      </c>
+      <c r="U355" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="V355" s="4" t="s">
+        <v>2595</v>
+      </c>
+      <c r="W355" s="4" t="s">
+        <v>2596</v>
+      </c>
+      <c r="X355" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y355" s="4" t="s">
+        <v>2597</v>
+      </c>
+      <c r="Z355" s="7" t="s">
+        <v>2598</v>
+      </c>
+      <c r="AA355" s="4" t="s">
+        <v>2589</v>
+      </c>
+    </row>
+    <row r="356" ht="22.5" customHeight="1">
+      <c r="A356" s="3">
+        <v>46210.54325797454</v>
+      </c>
+      <c r="B356" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="C356" s="5" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"S66")</f>
+        <v>S66</v>
+      </c>
+      <c r="D356" s="4" t="s">
+        <v>2599</v>
+      </c>
+      <c r="E356" s="4" t="s">
+        <v>2600</v>
+      </c>
+      <c r="F356" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G356" s="4" t="s">
+        <v>913</v>
+      </c>
+      <c r="H356" s="4" t="s">
+        <v>2600</v>
+      </c>
+      <c r="I356" s="4" t="s">
+        <v>2601</v>
+      </c>
+      <c r="J356" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="K356" s="4" t="s">
+        <v>2602</v>
+      </c>
+      <c r="L356" s="6">
+        <v>49597.0</v>
+      </c>
+      <c r="M356" s="4" t="s">
+        <v>2599</v>
+      </c>
+      <c r="N356" s="6">
+        <v>31618.0</v>
+      </c>
+      <c r="O356" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="P356" s="4" t="s">
+        <v>2603</v>
+      </c>
+      <c r="Q356" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="R356" s="7" t="s">
+        <v>2604</v>
+      </c>
+      <c r="S356" s="7" t="s">
+        <v>2604</v>
+      </c>
+      <c r="V356" s="4" t="s">
+        <v>1235</v>
+      </c>
+      <c r="W356" s="4" t="s">
+        <v>2605</v>
+      </c>
+      <c r="X356" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="Y356" s="7" t="s">
+        <v>2606</v>
+      </c>
+      <c r="Z356" s="4" t="s">
+        <v>2607</v>
+      </c>
+      <c r="AA356" s="4" t="s">
+        <v>2608</v>
+      </c>
+    </row>
+    <row r="357" ht="22.5" customHeight="1">
+      <c r="A357" s="3">
+        <v>46210.54662466435</v>
+      </c>
+      <c r="B357" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="C357" s="5" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"L89")</f>
+        <v>L89</v>
+      </c>
+      <c r="D357" s="4" t="s">
+        <v>2586</v>
+      </c>
+      <c r="E357" s="4" t="s">
+        <v>2587</v>
+      </c>
+      <c r="F357" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G357" s="4" t="s">
+        <v>2609</v>
+      </c>
+      <c r="H357" s="4" t="s">
+        <v>2587</v>
+      </c>
+      <c r="I357" s="4" t="s">
+        <v>2590</v>
+      </c>
+      <c r="J357" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="M357" s="4" t="s">
+        <v>2586</v>
+      </c>
+      <c r="N357" s="6">
+        <v>37902.0</v>
+      </c>
+      <c r="O357" s="4" t="s">
+        <v>674</v>
+      </c>
+      <c r="P357" s="4" t="s">
+        <v>2610</v>
+      </c>
+      <c r="Q357" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="R357" s="4" t="s">
+        <v>2611</v>
+      </c>
+      <c r="S357" s="4" t="s">
+        <v>2611</v>
+      </c>
+      <c r="V357" s="4" t="s">
+        <v>2595</v>
+      </c>
+      <c r="W357" s="4" t="s">
+        <v>2596</v>
+      </c>
+      <c r="X357" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="Y357" s="4" t="s">
+        <v>2597</v>
+      </c>
+      <c r="Z357" s="4">
+        <v>1.05057377100001E14</v>
+      </c>
+      <c r="AA357" s="4" t="s">
+        <v>2612</v>
+      </c>
+    </row>
+    <row r="358" ht="22.5" customHeight="1">
+      <c r="A358" s="10"/>
+      <c r="B358" s="10"/>
+      <c r="C358" s="10" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
         <v/>
       </c>
-      <c r="D355" s="10"/>
-      <c r="E355" s="10"/>
-      <c r="F355" s="10"/>
-      <c r="G355" s="10"/>
-      <c r="H355" s="10"/>
-      <c r="I355" s="10"/>
-      <c r="J355" s="10"/>
-      <c r="K355" s="10"/>
-      <c r="L355" s="10"/>
-      <c r="M355" s="10"/>
-      <c r="N355" s="10"/>
-      <c r="O355" s="10"/>
-      <c r="P355" s="10"/>
-      <c r="Q355" s="10"/>
-      <c r="R355" s="10"/>
-      <c r="S355" s="10"/>
-      <c r="T355" s="10"/>
-      <c r="U355" s="10"/>
-      <c r="V355" s="10"/>
-      <c r="W355" s="10"/>
-      <c r="X355" s="10"/>
-      <c r="Y355" s="10"/>
-      <c r="Z355" s="10"/>
-      <c r="AA355" s="10"/>
-      <c r="AB355" s="10"/>
-    </row>
-    <row r="356">
-      <c r="C356" s="11" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="357">
-      <c r="C357" s="11" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="358">
-      <c r="C358" s="11" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
-        <v/>
-      </c>
+      <c r="D358" s="10"/>
+      <c r="E358" s="10"/>
+      <c r="F358" s="10"/>
+      <c r="G358" s="10"/>
+      <c r="H358" s="10"/>
+      <c r="I358" s="10"/>
+      <c r="J358" s="10"/>
+      <c r="K358" s="10"/>
+      <c r="L358" s="10"/>
+      <c r="M358" s="10"/>
+      <c r="N358" s="10"/>
+      <c r="O358" s="10"/>
+      <c r="P358" s="10"/>
+      <c r="Q358" s="10"/>
+      <c r="R358" s="10"/>
+      <c r="S358" s="10"/>
+      <c r="T358" s="10"/>
+      <c r="U358" s="10"/>
+      <c r="V358" s="10"/>
+      <c r="W358" s="10"/>
+      <c r="X358" s="10"/>
+      <c r="Y358" s="10"/>
+      <c r="Z358" s="10"/>
+      <c r="AA358" s="10"/>
+      <c r="AB358" s="10"/>
     </row>
     <row r="359">
       <c r="C359" s="11" t="str">
@@ -36812,6 +37103,24 @@
     </row>
     <row r="454">
       <c r="C454" s="11" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="455">
+      <c r="C455" s="11" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="456">
+      <c r="C456" s="11" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="457">
+      <c r="C457" s="11" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
feat: async background PDF generation with progress polling — no more request timeout
</commit_message>
<xml_diff>
--- a/uploads/applicants.xlsx
+++ b/uploads/applicants.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6572" uniqueCount="2613">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6647" uniqueCount="2648">
   <si>
     <t>Timestamp</t>
   </si>
@@ -7857,6 +7857,111 @@
   </si>
   <si>
     <t>MUHAMMAD RASIM QURESHI</t>
+  </si>
+  <si>
+    <t>Muhammad Nasir</t>
+  </si>
+  <si>
+    <t>Nasir</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Jan Muhammad</t>
+  </si>
+  <si>
+    <t>BE9823713</t>
+  </si>
+  <si>
+    <t>Flat No 3, 2nd Floor, Latif Manzil, G.k ^/95 G. Allana Road, Kharadar, Karachi</t>
+  </si>
+  <si>
+    <t>03362271566</t>
+  </si>
+  <si>
+    <t>03062522562</t>
+  </si>
+  <si>
+    <t>Muhammad Sadiq</t>
+  </si>
+  <si>
+    <t>Brother in Law (Sala)</t>
+  </si>
+  <si>
+    <t>03082374329</t>
+  </si>
+  <si>
+    <t>PK95MPBL0128567140160630</t>
+  </si>
+  <si>
+    <t>Mohammad Nasir</t>
+  </si>
+  <si>
+    <t>hamm</t>
+  </si>
+  <si>
+    <t>Flat No,3, 2nd Floor, Latif Manzil, G.K 6/95 G. Allana Road, Kharadar, Karachi</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> PK95MPBL0128567140160630</t>
+  </si>
+  <si>
+    <t>Muhammad Sarfaraz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muhammad Sarfaraz </t>
+  </si>
+  <si>
+    <t>SARARAZ</t>
+  </si>
+  <si>
+    <t>ABDUL WAHID</t>
+  </si>
+  <si>
+    <t>BA5980544</t>
+  </si>
+  <si>
+    <t>42301-1054054-3</t>
+  </si>
+  <si>
+    <t>SHARFABAD , BAHADURABAD KARACHI</t>
+  </si>
+  <si>
+    <t>03219268789</t>
+  </si>
+  <si>
+    <t>42301-6523194-1</t>
+  </si>
+  <si>
+    <t>03212770389</t>
+  </si>
+  <si>
+    <t>PK02MEZN0001900104627782</t>
+  </si>
+  <si>
+    <t>42201-5851978-9</t>
+  </si>
+  <si>
+    <t>Shehroze Ahmed</t>
+  </si>
+  <si>
+    <t>Shehroze</t>
+  </si>
+  <si>
+    <t>TU1159783</t>
+  </si>
+  <si>
+    <t>House H92 Cantt Bazar Malir Cantt Karachi</t>
+  </si>
+  <si>
+    <t>+923009288085</t>
+  </si>
+  <si>
+    <t>42201-5569859-7</t>
+  </si>
+  <si>
+    <t>+923219288085</t>
+  </si>
+  <si>
+    <t>PK14MEZN0001200104506642</t>
   </si>
 </sst>
 </file>
@@ -8018,7 +8123,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:AB358" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:AB362" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="28">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Family Size  " id="2"/>
@@ -8373,26 +8478,26 @@
       </c>
       <c r="C2" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("ARRAYFORMULA(
-IF(D2:D457="""","""",
-IF(UPPER(TRIM(F2:F457))=""SHORT"",""S"",""L"")&amp;
+IF(D2:D461="""","""",
+IF(UPPER(TRIM(F2:F461))=""SHORT"",""S"",""L"")&amp;
 IF(
-UPPER(TRIM(F2:F457))=""SHORT"",
+UPPER(TRIM(F2:F461))=""SHORT"",
 MATCH(
-REGEXREPLACE(TO_TEXT(D2:D457),""[^0-9]"",""""),
+REGEXREPLACE(TO_TEXT(D2:D461),""[^0-9]"",""""),
 UNIQUE(
 FILTER(
-REGEXREPLACE(TO_TEXT(D2:D457),""[^0-9]"",""""),
-(D2:D457&lt;&gt;"""")*"&amp;"(UPPER(TRIM(F2:F457))=""SHORT"")
+REGEXREPLACE(TO_TEXT(D2:D461),""[^0-9]"",""""),
+(D2:D461&lt;&gt;"""")*"&amp;"(UPPER(TRIM(F2:F461))=""SHORT"")
 )
 ),
 0
 ),
 MATCH(
-REGEXREPLACE(TO_TEXT(D2:D457),""[^0-9]"",""""),
+REGEXREPLACE(TO_TEXT(D2:D461),""[^0-9]"",""""),
 UNIQUE(
 FILTER(
-REGEXREPLACE(TO_TEXT(D2:D457),""[^0-9]"",""""),
-(D2:D457&lt;&gt;"""")*(UPPER(TRIM(F2:F457))=""LONG"")
+REGEXREPLACE(TO_TEXT(D2:D461),""[^0-9]"",""""),
+(D2:D461&lt;&gt;"""")*(UPPER(TRIM(F2:F461))=""LONG"")
 )
 ),
 0
@@ -36499,61 +36604,349 @@
       </c>
     </row>
     <row r="358" ht="22.5" customHeight="1">
-      <c r="A358" s="10"/>
-      <c r="B358" s="10"/>
-      <c r="C358" s="10" t="str">
+      <c r="A358" s="3">
+        <v>46210.6284962037</v>
+      </c>
+      <c r="B358" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="C358" s="5" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"L90")</f>
+        <v>L90</v>
+      </c>
+      <c r="D358" s="4">
+        <v>4.230108783719E12</v>
+      </c>
+      <c r="E358" s="4" t="s">
+        <v>2613</v>
+      </c>
+      <c r="F358" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G358" s="4" t="s">
+        <v>2614</v>
+      </c>
+      <c r="H358" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I358" s="4" t="s">
+        <v>2615</v>
+      </c>
+      <c r="J358" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="K358" s="4" t="s">
+        <v>2616</v>
+      </c>
+      <c r="L358" s="6">
+        <v>46733.0</v>
+      </c>
+      <c r="M358" s="4">
+        <v>4.230108783719E12</v>
+      </c>
+      <c r="N358" s="6">
+        <v>22773.0</v>
+      </c>
+      <c r="O358" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="P358" s="4" t="s">
+        <v>2617</v>
+      </c>
+      <c r="Q358" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="R358" s="7" t="s">
+        <v>2618</v>
+      </c>
+      <c r="S358" s="7" t="s">
+        <v>2619</v>
+      </c>
+      <c r="V358" s="4" t="s">
+        <v>2620</v>
+      </c>
+      <c r="W358" s="4">
+        <v>4.200037664699E12</v>
+      </c>
+      <c r="X358" s="4" t="s">
+        <v>2621</v>
+      </c>
+      <c r="Y358" s="7" t="s">
+        <v>2622</v>
+      </c>
+      <c r="Z358" s="4" t="s">
+        <v>2623</v>
+      </c>
+      <c r="AA358" s="4" t="s">
+        <v>2624</v>
+      </c>
+    </row>
+    <row r="359" ht="22.5" customHeight="1">
+      <c r="A359" s="3">
+        <v>46210.63399229167</v>
+      </c>
+      <c r="B359" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="C359" s="5" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"L90")</f>
+        <v>L90</v>
+      </c>
+      <c r="D359" s="4">
+        <v>4.230108783719E12</v>
+      </c>
+      <c r="E359" s="4" t="s">
+        <v>2613</v>
+      </c>
+      <c r="F359" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G359" s="4" t="s">
+        <v>2625</v>
+      </c>
+      <c r="H359" s="4" t="s">
+        <v>2320</v>
+      </c>
+      <c r="I359" s="4" t="s">
+        <v>2613</v>
+      </c>
+      <c r="J359" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="M359" s="4">
+        <v>4.230108022556E12</v>
+      </c>
+      <c r="N359" s="6">
+        <v>25264.0</v>
+      </c>
+      <c r="O359" s="4" t="s">
+        <v>674</v>
+      </c>
+      <c r="P359" s="4" t="s">
+        <v>2626</v>
+      </c>
+      <c r="Q359" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="R359" s="7" t="s">
+        <v>2618</v>
+      </c>
+      <c r="S359" s="7" t="s">
+        <v>2619</v>
+      </c>
+      <c r="T359" s="4" t="s">
+        <v>2613</v>
+      </c>
+      <c r="U359" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="V359" s="4" t="s">
+        <v>2620</v>
+      </c>
+      <c r="W359" s="4">
+        <v>4.200037664699E12</v>
+      </c>
+      <c r="X359" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="Y359" s="7" t="s">
+        <v>2622</v>
+      </c>
+      <c r="Z359" s="4" t="s">
+        <v>2627</v>
+      </c>
+      <c r="AA359" s="4" t="s">
+        <v>2624</v>
+      </c>
+    </row>
+    <row r="360" ht="22.5" customHeight="1">
+      <c r="A360" s="3">
+        <v>46210.64301799769</v>
+      </c>
+      <c r="B360" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="C360" s="5" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"L72")</f>
+        <v>L72</v>
+      </c>
+      <c r="D360" s="4" t="s">
+        <v>2628</v>
+      </c>
+      <c r="E360" s="4" t="s">
+        <v>2629</v>
+      </c>
+      <c r="F360" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G360" s="4" t="s">
+        <v>2630</v>
+      </c>
+      <c r="H360" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="I360" s="4" t="s">
+        <v>2631</v>
+      </c>
+      <c r="J360" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="K360" s="4" t="s">
+        <v>2632</v>
+      </c>
+      <c r="L360" s="6">
+        <v>48812.0</v>
+      </c>
+      <c r="M360" s="4" t="s">
+        <v>2633</v>
+      </c>
+      <c r="N360" s="6">
+        <v>26699.0</v>
+      </c>
+      <c r="O360" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="P360" s="4" t="s">
+        <v>2634</v>
+      </c>
+      <c r="Q360" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="R360" s="7" t="s">
+        <v>2635</v>
+      </c>
+      <c r="S360" s="7" t="s">
+        <v>2635</v>
+      </c>
+      <c r="V360" s="4" t="s">
+        <v>2368</v>
+      </c>
+      <c r="W360" s="4" t="s">
+        <v>2636</v>
+      </c>
+      <c r="X360" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="Y360" s="7" t="s">
+        <v>2637</v>
+      </c>
+      <c r="Z360" s="4" t="s">
+        <v>2638</v>
+      </c>
+      <c r="AA360" s="4" t="s">
+        <v>1126</v>
+      </c>
+    </row>
+    <row r="361" ht="22.5" customHeight="1">
+      <c r="A361" s="3">
+        <v>46210.66009006945</v>
+      </c>
+      <c r="B361" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="C361" s="5" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"S67")</f>
+        <v>S67</v>
+      </c>
+      <c r="D361" s="4" t="s">
+        <v>2639</v>
+      </c>
+      <c r="E361" s="4" t="s">
+        <v>2640</v>
+      </c>
+      <c r="F361" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G361" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="H361" s="4" t="s">
+        <v>2641</v>
+      </c>
+      <c r="I361" s="4" t="s">
+        <v>2036</v>
+      </c>
+      <c r="J361" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="K361" s="4" t="s">
+        <v>2642</v>
+      </c>
+      <c r="L361" s="6">
+        <v>49143.0</v>
+      </c>
+      <c r="M361" s="4" t="s">
+        <v>2639</v>
+      </c>
+      <c r="N361" s="6">
+        <v>36618.0</v>
+      </c>
+      <c r="O361" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="P361" s="4" t="s">
+        <v>2643</v>
+      </c>
+      <c r="Q361" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="R361" s="4" t="s">
+        <v>2644</v>
+      </c>
+      <c r="S361" s="4" t="s">
+        <v>2644</v>
+      </c>
+      <c r="V361" s="4" t="s">
+        <v>2036</v>
+      </c>
+      <c r="W361" s="4" t="s">
+        <v>2645</v>
+      </c>
+      <c r="X361" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y361" s="4" t="s">
+        <v>2646</v>
+      </c>
+      <c r="Z361" s="4" t="s">
+        <v>2647</v>
+      </c>
+      <c r="AA361" s="4" t="s">
+        <v>2640</v>
+      </c>
+    </row>
+    <row r="362" ht="22.5" customHeight="1">
+      <c r="A362" s="10"/>
+      <c r="B362" s="10"/>
+      <c r="C362" s="10" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
         <v/>
       </c>
-      <c r="D358" s="10"/>
-      <c r="E358" s="10"/>
-      <c r="F358" s="10"/>
-      <c r="G358" s="10"/>
-      <c r="H358" s="10"/>
-      <c r="I358" s="10"/>
-      <c r="J358" s="10"/>
-      <c r="K358" s="10"/>
-      <c r="L358" s="10"/>
-      <c r="M358" s="10"/>
-      <c r="N358" s="10"/>
-      <c r="O358" s="10"/>
-      <c r="P358" s="10"/>
-      <c r="Q358" s="10"/>
-      <c r="R358" s="10"/>
-      <c r="S358" s="10"/>
-      <c r="T358" s="10"/>
-      <c r="U358" s="10"/>
-      <c r="V358" s="10"/>
-      <c r="W358" s="10"/>
-      <c r="X358" s="10"/>
-      <c r="Y358" s="10"/>
-      <c r="Z358" s="10"/>
-      <c r="AA358" s="10"/>
-      <c r="AB358" s="10"/>
-    </row>
-    <row r="359">
-      <c r="C359" s="11" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="360">
-      <c r="C360" s="11" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="361">
-      <c r="C361" s="11" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="362">
-      <c r="C362" s="11" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
-        <v/>
-      </c>
+      <c r="D362" s="10"/>
+      <c r="E362" s="10"/>
+      <c r="F362" s="10"/>
+      <c r="G362" s="10"/>
+      <c r="H362" s="10"/>
+      <c r="I362" s="10"/>
+      <c r="J362" s="10"/>
+      <c r="K362" s="10"/>
+      <c r="L362" s="10"/>
+      <c r="M362" s="10"/>
+      <c r="N362" s="10"/>
+      <c r="O362" s="10"/>
+      <c r="P362" s="10"/>
+      <c r="Q362" s="10"/>
+      <c r="R362" s="10"/>
+      <c r="S362" s="10"/>
+      <c r="T362" s="10"/>
+      <c r="U362" s="10"/>
+      <c r="V362" s="10"/>
+      <c r="W362" s="10"/>
+      <c r="X362" s="10"/>
+      <c r="Y362" s="10"/>
+      <c r="Z362" s="10"/>
+      <c r="AA362" s="10"/>
+      <c r="AB362" s="10"/>
     </row>
     <row r="363">
       <c r="C363" s="11" t="str">
@@ -37121,6 +37514,30 @@
     </row>
     <row r="457">
       <c r="C457" s="11" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="458">
+      <c r="C458" s="11" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="459">
+      <c r="C459" s="11" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="460">
+      <c r="C460" s="11" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="461">
+      <c r="C461" s="11" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
fix: auto-detect crashed Playwright browser and recreate with retry logic
</commit_message>
<xml_diff>
--- a/uploads/applicants.xlsx
+++ b/uploads/applicants.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6647" uniqueCount="2648">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6693" uniqueCount="2660">
   <si>
     <t>Timestamp</t>
   </si>
@@ -7962,6 +7962,42 @@
   </si>
   <si>
     <t>PK14MEZN0001200104506642</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E8, Gulshan Complex Phase-1 Gulistan-e-Jauhar Blk-19 Karachi </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gulistan-e-Jauhar Blk-19 Karachi </t>
+  </si>
+  <si>
+    <t>42000-1817579-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muhammad Irfan </t>
+  </si>
+  <si>
+    <t>Abdul Karim</t>
+  </si>
+  <si>
+    <t>LS1985791</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flat no 204 shazil comforts near hussani blood bank parsi colony </t>
+  </si>
+  <si>
+    <t>03322343414</t>
+  </si>
+  <si>
+    <t>03452343414</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fawad Abdul karim </t>
+  </si>
+  <si>
+    <t>03452343344</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Pk64 BAHL 1089 0081 0011 9801 4</t>
   </si>
 </sst>
 </file>
@@ -8123,7 +8159,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:AB362" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:AB365" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="28">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Family Size  " id="2"/>
@@ -8478,26 +8514,26 @@
       </c>
       <c r="C2" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("ARRAYFORMULA(
-IF(D2:D461="""","""",
-IF(UPPER(TRIM(F2:F461))=""SHORT"",""S"",""L"")&amp;
+IF(D2:D464="""","""",
+IF(UPPER(TRIM(F2:F464))=""SHORT"",""S"",""L"")&amp;
 IF(
-UPPER(TRIM(F2:F461))=""SHORT"",
+UPPER(TRIM(F2:F464))=""SHORT"",
 MATCH(
-REGEXREPLACE(TO_TEXT(D2:D461),""[^0-9]"",""""),
+REGEXREPLACE(TO_TEXT(D2:D464),""[^0-9]"",""""),
 UNIQUE(
 FILTER(
-REGEXREPLACE(TO_TEXT(D2:D461),""[^0-9]"",""""),
-(D2:D461&lt;&gt;"""")*"&amp;"(UPPER(TRIM(F2:F461))=""SHORT"")
+REGEXREPLACE(TO_TEXT(D2:D464),""[^0-9]"",""""),
+(D2:D464&lt;&gt;"""")*"&amp;"(UPPER(TRIM(F2:F464))=""SHORT"")
 )
 ),
 0
 ),
 MATCH(
-REGEXREPLACE(TO_TEXT(D2:D461),""[^0-9]"",""""),
+REGEXREPLACE(TO_TEXT(D2:D464),""[^0-9]"",""""),
 UNIQUE(
 FILTER(
-REGEXREPLACE(TO_TEXT(D2:D461),""[^0-9]"",""""),
-(D2:D461&lt;&gt;"""")*(UPPER(TRIM(F2:F461))=""LONG"")
+REGEXREPLACE(TO_TEXT(D2:D464),""[^0-9]"",""""),
+(D2:D464&lt;&gt;"""")*(UPPER(TRIM(F2:F464))=""LONG"")
 )
 ),
 0
@@ -36916,55 +36952,247 @@
       </c>
     </row>
     <row r="362" ht="22.5" customHeight="1">
-      <c r="A362" s="10"/>
-      <c r="B362" s="10"/>
-      <c r="C362" s="10" t="str">
+      <c r="A362" s="3">
+        <v>46210.77610878472</v>
+      </c>
+      <c r="B362" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="C362" s="5" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"L11")</f>
+        <v>L11</v>
+      </c>
+      <c r="D362" s="4">
+        <v>4.220106535795E12</v>
+      </c>
+      <c r="E362" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F362" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G362" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="H362" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="I362" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="J362" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="M362" s="4">
+        <v>4.220106535795E12</v>
+      </c>
+      <c r="N362" s="6">
+        <v>22605.0</v>
+      </c>
+      <c r="O362" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="P362" s="4" t="s">
+        <v>2648</v>
+      </c>
+      <c r="Q362" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="R362" s="7" t="s">
+        <v>397</v>
+      </c>
+      <c r="S362" s="7" t="s">
+        <v>397</v>
+      </c>
+      <c r="V362" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="W362" s="4">
+        <v>4.220168348347E12</v>
+      </c>
+      <c r="X362" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y362" s="7" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="363" ht="22.5" customHeight="1">
+      <c r="A363" s="3">
+        <v>46210.77931133102</v>
+      </c>
+      <c r="B363" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="C363" s="5" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"L11")</f>
+        <v>L11</v>
+      </c>
+      <c r="D363" s="4">
+        <v>4.220106535795E12</v>
+      </c>
+      <c r="E363" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="F363" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G363" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="H363" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="I363" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="J363" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="M363" s="4">
+        <v>4.220106535795E12</v>
+      </c>
+      <c r="N363" s="6">
+        <v>22605.0</v>
+      </c>
+      <c r="O363" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="P363" s="4" t="s">
+        <v>2649</v>
+      </c>
+      <c r="Q363" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="R363" s="7" t="s">
+        <v>397</v>
+      </c>
+      <c r="S363" s="7" t="s">
+        <v>397</v>
+      </c>
+      <c r="V363" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="W363" s="4">
+        <v>4.220168348347E12</v>
+      </c>
+      <c r="X363" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y363" s="7" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="364" ht="22.5" customHeight="1">
+      <c r="A364" s="3">
+        <v>46210.782794004626</v>
+      </c>
+      <c r="B364" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="C364" s="5" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"L91")</f>
+        <v>L91</v>
+      </c>
+      <c r="D364" s="4" t="s">
+        <v>2650</v>
+      </c>
+      <c r="E364" s="4" t="s">
+        <v>2651</v>
+      </c>
+      <c r="F364" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G364" s="4" t="s">
+        <v>2172</v>
+      </c>
+      <c r="H364" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I364" s="4" t="s">
+        <v>2652</v>
+      </c>
+      <c r="J364" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="K364" s="4" t="s">
+        <v>2653</v>
+      </c>
+      <c r="L364" s="6">
+        <v>46916.0</v>
+      </c>
+      <c r="M364" s="4">
+        <v>4.200018175791E12</v>
+      </c>
+      <c r="N364" s="6">
+        <v>27347.0</v>
+      </c>
+      <c r="O364" s="4" t="s">
+        <v>2134</v>
+      </c>
+      <c r="P364" s="4" t="s">
+        <v>2654</v>
+      </c>
+      <c r="Q364" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="R364" s="7" t="s">
+        <v>2655</v>
+      </c>
+      <c r="S364" s="7" t="s">
+        <v>2656</v>
+      </c>
+      <c r="V364" s="4" t="s">
+        <v>2657</v>
+      </c>
+      <c r="W364" s="4">
+        <v>4.200041696941E12</v>
+      </c>
+      <c r="X364" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="Y364" s="7" t="s">
+        <v>2658</v>
+      </c>
+      <c r="Z364" s="4" t="s">
+        <v>2659</v>
+      </c>
+      <c r="AA364" s="4" t="s">
+        <v>2164</v>
+      </c>
+    </row>
+    <row r="365" ht="22.5" customHeight="1">
+      <c r="A365" s="10"/>
+      <c r="B365" s="10"/>
+      <c r="C365" s="10" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
         <v/>
       </c>
-      <c r="D362" s="10"/>
-      <c r="E362" s="10"/>
-      <c r="F362" s="10"/>
-      <c r="G362" s="10"/>
-      <c r="H362" s="10"/>
-      <c r="I362" s="10"/>
-      <c r="J362" s="10"/>
-      <c r="K362" s="10"/>
-      <c r="L362" s="10"/>
-      <c r="M362" s="10"/>
-      <c r="N362" s="10"/>
-      <c r="O362" s="10"/>
-      <c r="P362" s="10"/>
-      <c r="Q362" s="10"/>
-      <c r="R362" s="10"/>
-      <c r="S362" s="10"/>
-      <c r="T362" s="10"/>
-      <c r="U362" s="10"/>
-      <c r="V362" s="10"/>
-      <c r="W362" s="10"/>
-      <c r="X362" s="10"/>
-      <c r="Y362" s="10"/>
-      <c r="Z362" s="10"/>
-      <c r="AA362" s="10"/>
-      <c r="AB362" s="10"/>
-    </row>
-    <row r="363">
-      <c r="C363" s="11" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="364">
-      <c r="C364" s="11" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="365">
-      <c r="C365" s="11" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
-        <v/>
-      </c>
+      <c r="D365" s="10"/>
+      <c r="E365" s="10"/>
+      <c r="F365" s="10"/>
+      <c r="G365" s="10"/>
+      <c r="H365" s="10"/>
+      <c r="I365" s="10"/>
+      <c r="J365" s="10"/>
+      <c r="K365" s="10"/>
+      <c r="L365" s="10"/>
+      <c r="M365" s="10"/>
+      <c r="N365" s="10"/>
+      <c r="O365" s="10"/>
+      <c r="P365" s="10"/>
+      <c r="Q365" s="10"/>
+      <c r="R365" s="10"/>
+      <c r="S365" s="10"/>
+      <c r="T365" s="10"/>
+      <c r="U365" s="10"/>
+      <c r="V365" s="10"/>
+      <c r="W365" s="10"/>
+      <c r="X365" s="10"/>
+      <c r="Y365" s="10"/>
+      <c r="Z365" s="10"/>
+      <c r="AA365" s="10"/>
+      <c r="AB365" s="10"/>
     </row>
     <row r="366">
       <c r="C366" s="11" t="str">
@@ -37538,6 +37766,24 @@
     </row>
     <row r="461">
       <c r="C461" s="11" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="462">
+      <c r="C462" s="11" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="463">
+      <c r="C463" s="11" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="464">
+      <c r="C464" s="11" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
         <v/>
       </c>

</xml_diff>